<commit_message>
feat(explorer): implement autonomous exploration with stealth, auto-login, and multi-tab support
</commit_message>
<xml_diff>
--- a/product Tester/templates/cnt_test_fkr.xlsx
+++ b/product Tester/templates/cnt_test_fkr.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
   </si>
   <si>
     <t>1. Nhập "Human" vào ô Search Apps.
-2. Click nút x bên phải Search Apps.</t>
+2. Xóa "Human" trong ô Search Apps.</t>
   </si>
   <si>
     <t>Chỉ hiển thị card "Human Resource Management".</t>
@@ -95,8 +95,8 @@
     <t>Kiểm tra điều hướng khi click vào App</t>
   </si>
   <si>
-    <t>1. Click vào card "Human Resource Managemen".
-2. Đóng tab "Human Resource Managemen".</t>
+    <t>1. Click "Human Resource Managemen".
+2. Đóng cửa số "Human Resource Managemen".</t>
   </si>
   <si>
     <t>Hệ thống chuyển hướng đúng sang trang Human Resource Management.</t>
@@ -106,7 +106,7 @@
   </si>
   <si>
     <t>1. Click vào card "Ticket Management".
-2. Đóng tab "Ticket Management".</t>
+2. Đóng cửa sổ "Ticket Management".</t>
   </si>
   <si>
     <t>Hệ thống chuyển hướng đúng sang trang Ticket Management.</t>
@@ -116,7 +116,7 @@
   </si>
   <si>
     <t>1. Click vào card "SLA".
-2. 2. Đóng tab "SLA".</t>
+2. Đóng cửa sổ "SLA".</t>
   </si>
   <si>
     <t>Hệ thống chuyển hướng đúng sang trang SLA.</t>
@@ -128,15 +128,16 @@
     <t>Kiểm tra chức năng thu gọn/mở rộng sơ đồ</t>
   </si>
   <si>
-    <t>1. Thực hiện TC-04 . 
-2. Click tab "Department Graph".
-3.  Click  (-) dưới node FKR (N/A) màu đỏ</t>
-  </si>
-  <si>
-    <t>Node con của phòng ban đó sẽ ẩn đi/hiện lại.</t>
-  </si>
-  <si>
-    <t>TC4-Passed</t>
+    <t>1. Click "Human Resource Managemen". 
+2. Click "Menu"
+3. Click  "Departments".
+4. Click "Employees"
+5. Click "Advance Settings"
+6. Click "Job title"
+7. Click "Skill"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chuyển đổi giữa các tab </t>
   </si>
   <si>
     <t>TC-08</t>
@@ -151,6 +152,9 @@
   </si>
   <si>
     <t>Chuyển từ dạng sơ đồ sang dạng bảng (Table/List)</t>
+  </si>
+  <si>
+    <t>TC4-Passed</t>
   </si>
   <si>
     <t>TC-09</t>
@@ -1679,7 +1683,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="43.2" spans="1:5">
+    <row r="8" ht="100.8" spans="1:5">
       <c r="A8" s="9" t="s">
         <v>28</v>
       </c>
@@ -1693,24 +1697,24 @@
         <v>31</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="43.2" spans="1:5">
       <c r="A9" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="C9" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E9" s="12" t="s">
         <v>36</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" ht="28.8" spans="1:5">
@@ -1727,7 +1731,7 @@
         <v>40</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" ht="28.8" spans="1:5">

</xml_diff>